<commit_message>
fixed signature inconsistency issue
</commit_message>
<xml_diff>
--- a/artifacts/output/output.xlsx
+++ b/artifacts/output/output.xlsx
@@ -28,12 +28,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,9 +54,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,11 +443,6 @@
           <t>Daily Spending (£)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -479,11 +482,6 @@
       <c r="C4" t="n">
         <v>89.53</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Gift</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -497,11 +495,6 @@
       <c r="C5" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Gift</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -515,11 +508,6 @@
       <c r="C6" t="n">
         <v>61.14</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -533,11 +521,6 @@
       <c r="C7" t="n">
         <v>92.15000000000001</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Bus fare</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -551,22 +534,17 @@
       <c r="C8" t="n">
         <v>76.3</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Coffee</t>
-        </is>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>45969</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="3" t="n">
         <v>116.58</v>
       </c>
     </row>
@@ -582,11 +560,6 @@
       <c r="C10" t="n">
         <v>32.59</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Groceries</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -600,11 +573,6 @@
       <c r="C11" t="n">
         <v>58.96</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Clothes</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -618,11 +586,6 @@
       <c r="C12" t="n">
         <v>56.22</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Groceries</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -636,11 +599,6 @@
       <c r="C13" t="n">
         <v>93.13</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Gift</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -654,11 +612,6 @@
       <c r="C14" t="n">
         <v>67.38</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Bus fare</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -672,11 +625,6 @@
       <c r="C15" t="n">
         <v>73.28</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Groceries</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -690,264 +638,139 @@
       <c r="C16" t="n">
         <v>67.03</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
       <c r="C17" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
       <c r="C18" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
       <c r="C19" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
       <c r="C20" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n"/>
       <c r="C21" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>45977</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Entertainment</t>
-        </is>
-      </c>
+      <c r="A22" s="1" t="n"/>
       <c r="C22" t="n">
-        <v>51.77</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Dinner</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>45978</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
+      <c r="A23" s="1" t="n"/>
       <c r="C23" t="n">
-        <v>101.05</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Groceries</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>45979</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
+      <c r="A24" s="1" t="n"/>
       <c r="C24" t="n">
-        <v>42.52</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Dinner</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>45980</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
+      <c r="A25" s="1" t="n"/>
       <c r="C25" t="n">
-        <v>107.96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>45981</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
+      <c r="A26" s="1" t="n"/>
       <c r="C26" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Coffee</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>45982</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Shopping</t>
-        </is>
-      </c>
+      <c r="A27" s="1" t="n"/>
       <c r="C27" t="n">
-        <v/>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Coffee</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>45983</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
+      <c r="A28" s="1" t="n"/>
       <c r="C28" t="n">
-        <v>38.45</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Cinema</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>45984</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
+      <c r="A29" s="1" t="n"/>
       <c r="C29" t="n">
-        <v>115.04</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
-        <v>45985</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
+      <c r="A30" s="1" t="n"/>
       <c r="C30" t="n">
-        <v>71.52</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Dinner</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
-        <v>45986</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Shopping</t>
-        </is>
-      </c>
+      <c r="A31" s="1" t="n"/>
       <c r="C31" t="n">
-        <v>111.18</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>45987</v>
+        <v>45977</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Entertainment</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>102.98</v>
+        <v>51.77</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>45988</v>
+        <v>45978</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Entertainment</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>57.13</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Groceries</t>
-        </is>
+        <v>101.05</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>45989</v>
+        <v>45979</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Entertainment</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Dinner</t>
-        </is>
+        <v>42.52</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>45990</v>
+        <v>45980</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -955,92 +778,272 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>99.25</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Gift</t>
-        </is>
+        <v>107.96</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
+        <v>45981</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>22.64</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>45983</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>38.45</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>45984</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>115.04</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>71.52</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>45986</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>111.18</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>45987</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>102.98</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>45988</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>57.13</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>45989</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>45990</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>99.25</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
         <v>45991</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>Shopping</t>
         </is>
       </c>
-      <c r="C36" t="n">
+      <c r="C46" t="n">
         <v>35.74</v>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Dinner</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="n"/>
-      <c r="C37" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="n"/>
-      <c r="C38" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="n"/>
-      <c r="C39" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="n"/>
-      <c r="C40" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="n"/>
-      <c r="C41" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n"/>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n"/>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n"/>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n"/>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n"/>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n"/>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n"/>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n"/>
+      <c r="C54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n"/>
+      <c r="C55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n"/>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n"/>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n"/>
+      <c r="C58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n"/>
+      <c r="C59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n"/>
+      <c r="C60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n"/>
+      <c r="C61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>Total Spending (£)</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B64" t="n">
         <v>2023.75</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>Average Daily Spending (£)</t>
         </is>
       </c>
-      <c r="B45" t="n">
-        <v>69.78448275862068</v>
+      <c r="B65" t="n">
+        <v>33.72916666666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
simplified the sheethero logic
</commit_message>
<xml_diff>
--- a/artifacts/output/output.xlsx
+++ b/artifacts/output/output.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,6 +443,11 @@
           <t>Daily Spending (£)</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -482,6 +487,11 @@
       <c r="C4" t="n">
         <v>89.53</v>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -495,6 +505,11 @@
       <c r="C5" t="n">
         <v>0</v>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -508,6 +523,11 @@
       <c r="C6" t="n">
         <v>61.14</v>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -521,6 +541,11 @@
       <c r="C7" t="n">
         <v>92.15000000000001</v>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Bus fare</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -534,6 +559,11 @@
       <c r="C8" t="n">
         <v>76.3</v>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Coffee</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -547,6 +577,7 @@
       <c r="C9" s="3" t="n">
         <v>116.58</v>
       </c>
+      <c r="D9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -560,6 +591,11 @@
       <c r="C10" t="n">
         <v>32.59</v>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -573,6 +609,11 @@
       <c r="C11" t="n">
         <v>58.96</v>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Clothes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -586,6 +627,11 @@
       <c r="C12" t="n">
         <v>56.22</v>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -599,6 +645,11 @@
       <c r="C13" t="n">
         <v>93.13</v>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -612,6 +663,11 @@
       <c r="C14" t="n">
         <v>67.38</v>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Bus fare</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -625,6 +681,11 @@
       <c r="C15" t="n">
         <v>73.28</v>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -638,95 +699,100 @@
       <c r="C16" t="n">
         <v>67.03</v>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
       <c r="C17" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
       <c r="C18" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
       <c r="C19" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
       <c r="C20" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n"/>
       <c r="C21" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n"/>
       <c r="C22" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n"/>
       <c r="C23" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n"/>
       <c r="C24" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n"/>
       <c r="C25" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n"/>
       <c r="C26" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n"/>
       <c r="C27" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n"/>
       <c r="C28" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n"/>
       <c r="C29" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n"/>
       <c r="C30" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
       <c r="C31" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -741,6 +807,11 @@
       <c r="C32" t="n">
         <v>51.77</v>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -754,6 +825,11 @@
       <c r="C33" t="n">
         <v>101.05</v>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -767,6 +843,11 @@
       <c r="C34" t="n">
         <v>42.52</v>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -793,6 +874,11 @@
       <c r="C36" t="n">
         <v>22.64</v>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Coffee</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -806,6 +892,11 @@
       <c r="C37" t="n">
         <v>0</v>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Coffee</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -819,6 +910,11 @@
       <c r="C38" t="n">
         <v>38.45</v>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Cinema</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -845,6 +941,11 @@
       <c r="C40" t="n">
         <v>71.52</v>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -858,6 +959,11 @@
       <c r="C41" t="n">
         <v>111.18</v>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -884,6 +990,11 @@
       <c r="C43" t="n">
         <v>57.13</v>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -897,6 +1008,11 @@
       <c r="C44" t="n">
         <v>32.5</v>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -910,6 +1026,11 @@
       <c r="C45" t="n">
         <v>99.25</v>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -923,95 +1044,100 @@
       <c r="C46" t="n">
         <v>35.74</v>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n"/>
       <c r="C47" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n"/>
       <c r="C48" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n"/>
       <c r="C49" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n"/>
       <c r="C50" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n"/>
       <c r="C51" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n"/>
       <c r="C52" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n"/>
       <c r="C53" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n"/>
       <c r="C54" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n"/>
       <c r="C55" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n"/>
       <c r="C56" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n"/>
       <c r="C57" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n"/>
       <c r="C58" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n"/>
       <c r="C59" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n"/>
       <c r="C60" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n"/>
       <c r="C61" t="n">
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -1043,7 +1169,29 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>33.72916666666666</v>
+        <v>67.45833333333333</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Max Spending Day(s)</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2025-11-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Max Spending Amount (£)</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>116.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>